<commit_message>
Add detailed timing data: unlock dates, sell velocity, time-to-first-sell
- sample_data.py: generate_sample_timing() produces per-wallet timing
  (unlock date/block/tx, first sell date, last activity, sell velocity,
  days active, # sell txs, Arkham labels, data source attribution)
- dashboard.py: 2 new charts (Sell Velocity bar, Time to First Sell bar),
  6 KPI cards (added avg velocity + total sell txs), 15-column table with
  full timing breakdown (unlock date, first sell, last activity, # txs,
  velocity, days active, source)
- main.py: wire timing data into tracking DataFrame for both outputs

https://claude.ai/code/session_01LdiCcWEnxFYsTuoFs5FhHg
</commit_message>
<xml_diff>
--- a/xpl_unlock_report.xlsx
+++ b/xpl_unlock_report.xlsx
@@ -550,7 +550,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-02-24 07:14 UTC</t>
+          <t>Generated 2026-02-24 16:06 UTC</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Arkham Intel (Ecosystem Development Fund)</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="I3" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Arkham Intel (Plasma Foundation)</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Arkham Intel (Early Investor B)</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="I5" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="I7" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Arkham Intel (Early Investor A)</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="I9" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Arkham Intel (Team Vesting Contract)</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="I11" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="I13" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="I15" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="I17" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="I19" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="I21" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="I23" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="I25" s="20" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>Plasma RPC (block scan)</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Plasma RPC / PlasmaScan</t>
+          <t>PlasmaScan API + Plasma RPC</t>
         </is>
       </c>
     </row>

</xml_diff>